<commit_message>
Odvolávky: směny podle výkonu kategorií, Excel se seskupenými řádky
Plánování → Kapacity má výkon za směnu podle projektu a kategorie
(řádek pro každý projekt a kategorii z mapování; Kapacity.xlsx, list
Výkon kategorií). Odvolávky (Přehled po projektech i Aktuální) mají
zaškrtávátko Zobrazit směny: pod každým řádkem kusů řádek směn = kusy
÷ výkon kategorie; součty jen z dílů s výkonem, chybějící výkon je
označený a vypsaný pod tabulkou.

Excel pro vedení: list Přehled s celým stromem, sloupci Ks / směna
a Jednotka a řádky ks a sm.; řádky jsou v Excelu seskupené (−/+, 1 2 3)
a sbalené jako v aplikaci. List Díly je seskupený pod projekt
a kategorii s řádky součtů. Seskupení dělá doplněk knihovny
write-excel-file (outlineLevel, sheetPr/outlinePr).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XrKYg9HPRfNVPS3U3EtT1P
</commit_message>
<xml_diff>
--- a/sample-data/Plan/Kapacity.xlsx
+++ b/sample-data/Plan/Kapacity.xlsx
@@ -9,6 +9,7 @@
     <sheet r:id="rId1" sheetId="1" name="Linky"/>
     <sheet r:id="rId2" sheetId="2" name="Destinace"/>
     <sheet r:id="rId3" sheetId="3" name="Směny"/>
+    <sheet r:id="rId4" sheetId="4" name="Výkon kategorií"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -76,6 +77,18 @@
   </si>
   <si>
     <t>Ranní směna od</t>
+  </si>
+  <si>
+    <t>Kategorie</t>
+  </si>
+  <si>
+    <t>DP</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>GB</t>
   </si>
 </sst>
 </file>
@@ -285,4 +298,55 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4">
+        <v>240</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>